<commit_message>
fig dutch report update
</commit_message>
<xml_diff>
--- a/input/group_names_to_translate.xlsx
+++ b/input/group_names_to_translate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\20204133\Documents\GitHub\PONG_DCE\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04E5434-DB39-4FE0-955F-A9EFE0EF291E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F1231D-34C2-43EC-9E13-21925EBC300B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{E6096B9A-0410-4633-B791-B641E9FD97DC}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="93">
   <si>
     <t>group</t>
   </si>
@@ -537,104 +537,148 @@
     <t>Bewoners zijn zelf in staat om te bepalen hoe ze van het gas afgaan.</t>
   </si>
   <si>
+    <t>Ik ben iemand die zich klimaatbewust gedraagt.</t>
+  </si>
+  <si>
+    <t>Negatief</t>
+  </si>
+  <si>
+    <t>Positief</t>
+  </si>
+  <si>
+    <t>Ik woon graag in mijn gemeente.</t>
+  </si>
+  <si>
+    <t>Ik woon graag in mijn wijk.</t>
+  </si>
+  <si>
+    <t>De prijzen voor warmtenetten moeten zo veel mogelijk gelijk zijn voor iedereen in de gemeente.</t>
+  </si>
+  <si>
+    <t>Ik denk dat de gemeente alles over de warmtetransitie al heeft besloten, mijn mening doet er niet toe.</t>
+  </si>
+  <si>
+    <t>Gemeente</t>
+  </si>
+  <si>
+    <t>Medemblik</t>
+  </si>
+  <si>
+    <t>Hoorn</t>
+  </si>
+  <si>
+    <t>Education 0 - Other</t>
+  </si>
+  <si>
+    <t>Education 1 - VMBO or lower</t>
+  </si>
+  <si>
+    <t>Education 2 - HAVO</t>
+  </si>
+  <si>
+    <t>Education 4 - master or higher</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>HAVO</t>
+  </si>
+  <si>
+    <t>Bachelor</t>
+  </si>
+  <si>
+    <t>Education 3 - bachelor</t>
+  </si>
+  <si>
+    <t>Construction year 1 - 1945 or before</t>
+  </si>
+  <si>
+    <t>Construction year 3 - 1991-2005</t>
+  </si>
+  <si>
+    <t>Construction year 2 - 1946-1990</t>
+  </si>
+  <si>
+    <t>Construction year 4 - 2006-2025</t>
+  </si>
+  <si>
+    <t>1946-1990</t>
+  </si>
+  <si>
+    <t>1991-2005</t>
+  </si>
+  <si>
+    <t>2006-2025</t>
+  </si>
+  <si>
+    <t>1945 of eerder</t>
+  </si>
+  <si>
+    <t>Bouwjaar</t>
+  </si>
+  <si>
+    <t>Opleiding</t>
+  </si>
+  <si>
+    <t>Master+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vmbo- </t>
+  </si>
+  <si>
+    <r>
+      <t>"People PONG positive"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFBBBEBF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA5D6FF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>"desc_In your opinion, how many people are positive about phasing out natural gas?"</t>
+    </r>
+  </si>
+  <si>
+    <t>People PONG positive 1 - Less than half</t>
+  </si>
+  <si>
+    <t>People PONG positive 2 - About half</t>
+  </si>
+  <si>
+    <t>People PONG positive 3 - More than half</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meer dan de helft </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ongeveer de helft </t>
+  </si>
+  <si>
+    <t>Minder dan de helft</t>
+  </si>
+  <si>
     <t>De gemeente is het beste in staat om te bepalen wat de meest goedkopen manier is om van het gas af te gaan.</t>
   </si>
   <si>
-    <t>Ik ben iemand die zich klimaatbewust gedraagt.</t>
-  </si>
-  <si>
-    <t>Negatief</t>
-  </si>
-  <si>
-    <t>Positief</t>
-  </si>
-  <si>
-    <t>Ik woon graag in mijn gemeente.</t>
-  </si>
-  <si>
-    <t>Ik woon graag in mijn wijk.</t>
-  </si>
-  <si>
-    <t>De prijzen voor warmtenetten moeten zo veel mogelijk gelijk zijn voor iedereen in de gemeente.</t>
-  </si>
-  <si>
-    <t>Ik denk dat de gemeente alles over de warmtetransitie al heeft besloten, mijn mening doet er niet toe.</t>
-  </si>
-  <si>
-    <t>Gemeente</t>
-  </si>
-  <si>
-    <t>Medemblik</t>
-  </si>
-  <si>
-    <t>Hoorn</t>
-  </si>
-  <si>
-    <t>Education 0 - Other</t>
-  </si>
-  <si>
-    <t>Education 1 - VMBO or lower</t>
-  </si>
-  <si>
-    <t>Education 2 - HAVO</t>
-  </si>
-  <si>
-    <t>Education 4 - master or higher</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>HAVO</t>
-  </si>
-  <si>
-    <t>Bachelor</t>
-  </si>
-  <si>
-    <t>Education 3 - bachelor</t>
-  </si>
-  <si>
-    <t>Construction year 1 - 1945 or before</t>
-  </si>
-  <si>
-    <t>Construction year 3 - 1991-2005</t>
-  </si>
-  <si>
-    <t>Construction year 2 - 1946-1990</t>
-  </si>
-  <si>
-    <t>Construction year 4 - 2006-2025</t>
-  </si>
-  <si>
-    <t>1946-1990</t>
-  </si>
-  <si>
-    <t>1991-2005</t>
-  </si>
-  <si>
-    <t>2006-2025</t>
-  </si>
-  <si>
-    <t>1945 of eerder</t>
-  </si>
-  <si>
-    <t>Bouwjaar</t>
-  </si>
-  <si>
-    <t>Opleiding</t>
-  </si>
-  <si>
-    <t>Master+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vmbo- </t>
+    <t xml:space="preserve">Hoeveel mensen in uw wijk zijn naar uw mening positief over afstappen van aardgas? </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -798,6 +842,24 @@
       <color theme="1"/>
       <name val="Noto Sans"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFBBBEBF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7EE787"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFA5D6FF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1147,7 +1209,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1158,6 +1220,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1533,12 +1598,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCAA32F7-7A0B-48F4-AC99-865C359ED2EF}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="3" max="3" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="99.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.85546875" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -1619,7 +1684,7 @@
         <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="D5" t="s">
         <v>50</v>
@@ -1636,7 +1701,7 @@
         <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
         <v>51</v>
@@ -1653,7 +1718,7 @@
         <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
         <v>52</v>
@@ -1670,7 +1735,7 @@
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
         <v>50</v>
@@ -1687,7 +1752,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
         <v>51</v>
@@ -1704,7 +1769,7 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D10" t="s">
         <v>52</v>
@@ -1724,7 +1789,7 @@
         <v>47</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>35</v>
@@ -1758,7 +1823,7 @@
         <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>35</v>
@@ -1772,7 +1837,7 @@
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
         <v>50</v>
@@ -1789,7 +1854,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
         <v>51</v>
@@ -1806,7 +1871,7 @@
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
         <v>52</v>
@@ -1823,7 +1888,7 @@
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
         <v>50</v>
@@ -1840,7 +1905,7 @@
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D18" t="s">
         <v>51</v>
@@ -1857,7 +1922,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D19" t="s">
         <v>52</v>
@@ -1874,7 +1939,7 @@
         <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D20" t="s">
         <v>50</v>
@@ -1891,7 +1956,7 @@
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D21" t="s">
         <v>51</v>
@@ -1908,7 +1973,7 @@
         <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D22" t="s">
         <v>52</v>
@@ -1928,7 +1993,7 @@
         <v>48</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>39</v>
@@ -1962,7 +2027,7 @@
         <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>39</v>
@@ -1974,10 +2039,10 @@
       </c>
       <c r="B26" s="2"/>
       <c r="C26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>40</v>
@@ -1989,10 +2054,10 @@
       </c>
       <c r="B27" s="2"/>
       <c r="C27" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" t="s">
         <v>62</v>
-      </c>
-      <c r="D27" t="s">
-        <v>63</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>40</v>
@@ -2004,7 +2069,7 @@
       </c>
       <c r="B28" s="2"/>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>46</v>
@@ -2021,7 +2086,7 @@
         <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D29" t="s">
         <v>50</v>
@@ -2038,7 +2103,7 @@
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D30" t="s">
         <v>51</v>
@@ -2055,7 +2120,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D31" t="s">
         <v>52</v>
@@ -2066,101 +2131,143 @@
     </row>
     <row r="32" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A32" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D32" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A33" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C33" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A34" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A35" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D35" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A36" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D36" t="s">
         <v>82</v>
       </c>
-      <c r="D32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="20.25" x14ac:dyDescent="0.45">
-      <c r="A33" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D33" s="5" t="s">
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C39" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A41" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D41" t="s">
+        <v>88</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="20.25" x14ac:dyDescent="0.45">
-      <c r="A34" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D34" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="20.25" x14ac:dyDescent="0.45">
-      <c r="A35" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="20.25" x14ac:dyDescent="0.45">
-      <c r="A36" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D36" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C37" t="s">
-        <v>81</v>
-      </c>
-      <c r="D37" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C38" t="s">
-        <v>81</v>
-      </c>
-      <c r="D38" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C39" t="s">
-        <v>81</v>
-      </c>
-      <c r="D39" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C40" t="s">
-        <v>81</v>
-      </c>
-      <c r="D40" t="s">
-        <v>79</v>
+    <row r="42" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A42" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D42" t="s">
+        <v>89</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="20.25" x14ac:dyDescent="0.45">
+      <c r="A43" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D43" t="s">
+        <v>90</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>